<commit_message>
numerous enhancement of python code examples
</commit_message>
<xml_diff>
--- a/Py_functionality_libs/py_excel/test.xlsx
+++ b/Py_functionality_libs/py_excel/test.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>Hello World2</t>
+    <t>Hello World27lul08</t>
   </si>
 </sst>
 </file>
@@ -74,7 +74,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>882906</xdr:colOff>
+      <xdr:colOff>749556</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>25519</xdr:rowOff>
     </xdr:to>
@@ -93,7 +93,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1381125" y="0"/>
+          <a:off x="1447800" y="0"/>
           <a:ext cx="4978656" cy="2311519"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -394,8 +394,8 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="4" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
+    <col min="2" max="4" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">

</xml_diff>

<commit_message>
Enhance Python examples and add SQL solutions July 2026 week 1 (#197)
* enumerate example
* Java Post Project
* SQL leetcode 570
* python leetcode 34
* python leetcode 36 - partly
* python leetcode 36 - partly
* python leetcode 36 - passed improved
* python insert into the beginning of the list
* leetcode python 39 in progress
* pytest_bdd example with class
* python_completing_time
* numerous enhancement of python code examples
* decorator wrapper example plus code black . improving
</commit_message>
<xml_diff>
--- a/Py_functionality_libs/py_excel/test.xlsx
+++ b/Py_functionality_libs/py_excel/test.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>Hello World2</t>
+    <t>Hello World27lul08</t>
   </si>
 </sst>
 </file>
@@ -74,7 +74,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>882906</xdr:colOff>
+      <xdr:colOff>749556</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>25519</xdr:rowOff>
     </xdr:to>
@@ -93,7 +93,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1381125" y="0"/>
+          <a:off x="1447800" y="0"/>
           <a:ext cx="4978656" cy="2311519"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -394,8 +394,8 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="4" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
+    <col min="2" max="4" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">

</xml_diff>